<commit_message>
add more file type tp parse
</commit_message>
<xml_diff>
--- a/invoice_automation/clients/northsky_comm/downloads/PROCESSED/invoice_load_001.xlsx
+++ b/invoice_automation/clients/northsky_comm/downloads/PROCESSED/invoice_load_001.xlsx
@@ -543,7 +543,7 @@
     <outlinePr summaryBelow="0"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:DL14"/>
+  <dimension ref="A1:DL12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.5"/>
   <cols>
     <col width="26" bestFit="1" customWidth="1" style="6" min="1" max="1"/>
@@ -1987,7 +1987,7 @@
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>06/08/26</t>
+          <t>06/09/26</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
@@ -2048,7 +2048,7 @@
       <c r="D8" t="inlineStr"/>
       <c r="E8" t="inlineStr">
         <is>
-          <t>1005638</t>
+          <t>5-31-26</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
@@ -2058,7 +2058,7 @@
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>06/08/26</t>
+          <t>06/09/26</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
@@ -2068,7 +2068,7 @@
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>DITCH WITCH Invoice 1005638</t>
+          <t>DITCH WITCH Invoice 5-31-26</t>
         </is>
       </c>
       <c r="J8" t="inlineStr">
@@ -2123,17 +2123,17 @@
       <c r="D9" t="inlineStr"/>
       <c r="E9" t="inlineStr">
         <is>
-          <t>154281</t>
+          <t>134882087</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>04/25/2025</t>
+          <t>05/27/26</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>06/08/26</t>
+          <t>06/09/26</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
@@ -2143,7 +2143,7 @@
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>VALVOLINE Invoice 154281</t>
+          <t>FLEETPRIDE Invoice 134882087</t>
         </is>
       </c>
       <c r="J9" t="inlineStr">
@@ -2151,8 +2151,10 @@
           <t>USD</t>
         </is>
       </c>
-      <c r="K9" t="n">
-        <v>300.78</v>
+      <c r="K9" t="inlineStr">
+        <is>
+          <t>1148.98</t>
+        </is>
       </c>
       <c r="BS9" t="inlineStr"/>
       <c r="BT9" t="inlineStr">
@@ -2166,8 +2168,10 @@
           <t>S</t>
         </is>
       </c>
-      <c r="BW9" t="n">
-        <v>300.78</v>
+      <c r="BW9" t="inlineStr">
+        <is>
+          <t>1148.98</t>
+        </is>
       </c>
       <c r="BX9" t="inlineStr">
         <is>
@@ -2194,17 +2198,17 @@
       <c r="D10" t="inlineStr"/>
       <c r="E10" t="inlineStr">
         <is>
-          <t>134882087</t>
+          <t>882430</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>05/27/26</t>
+          <t>05/29/2026</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>06/08/26</t>
+          <t>06/09/26</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
@@ -2214,7 +2218,7 @@
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>FLEETPRIDE Invoice 134882087</t>
+          <t xml:space="preserve"> Invoice 882430</t>
         </is>
       </c>
       <c r="J10" t="inlineStr">
@@ -2222,10 +2226,8 @@
           <t>USD</t>
         </is>
       </c>
-      <c r="K10" t="inlineStr">
-        <is>
-          <t>1148.98</t>
-        </is>
+      <c r="K10" t="n">
+        <v>64</v>
       </c>
       <c r="BS10" t="inlineStr"/>
       <c r="BT10" t="inlineStr">
@@ -2239,10 +2241,8 @@
           <t>S</t>
         </is>
       </c>
-      <c r="BW10" t="inlineStr">
-        <is>
-          <t>1148.98</t>
-        </is>
+      <c r="BW10" t="n">
+        <v>64</v>
       </c>
       <c r="BX10" t="inlineStr">
         <is>
@@ -2269,17 +2269,17 @@
       <c r="D11" t="inlineStr"/>
       <c r="E11" t="inlineStr">
         <is>
-          <t>882430</t>
+          <t>99923980</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>05/29/2026</t>
+          <t>05/22/2026</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>06/08/26</t>
+          <t>06/09/26</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
@@ -2289,7 +2289,7 @@
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t xml:space="preserve"> Invoice 882430</t>
+          <t>JIFFY LUBE Invoice 99923980</t>
         </is>
       </c>
       <c r="J11" t="inlineStr">
@@ -2298,7 +2298,7 @@
         </is>
       </c>
       <c r="K11" t="n">
-        <v>64</v>
+        <v>143.62</v>
       </c>
       <c r="BS11" t="inlineStr"/>
       <c r="BT11" t="inlineStr">
@@ -2313,7 +2313,7 @@
         </is>
       </c>
       <c r="BW11" t="n">
-        <v>64</v>
+        <v>143.62</v>
       </c>
       <c r="BX11" t="inlineStr">
         <is>
@@ -2340,17 +2340,17 @@
       <c r="D12" t="inlineStr"/>
       <c r="E12" t="inlineStr">
         <is>
-          <t>99923980</t>
+          <t>167142</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>05/22/2026</t>
+          <t>01/20/2026</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>06/08/26</t>
+          <t>06/09/26</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
@@ -2360,7 +2360,7 @@
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>JIFFY LUBE Invoice 99923980</t>
+          <t>VALVOLINE INSTANT OIL CHANGE Invoice 167142</t>
         </is>
       </c>
       <c r="J12" t="inlineStr">
@@ -2369,7 +2369,7 @@
         </is>
       </c>
       <c r="K12" t="n">
-        <v>143.62</v>
+        <v>116.21</v>
       </c>
       <c r="BS12" t="inlineStr"/>
       <c r="BT12" t="inlineStr">
@@ -2384,7 +2384,7 @@
         </is>
       </c>
       <c r="BW12" t="n">
-        <v>143.62</v>
+        <v>116.21</v>
       </c>
       <c r="BX12" t="inlineStr">
         <is>
@@ -2393,148 +2393,6 @@
       </c>
       <c r="BY12" t="inlineStr"/>
       <c r="CA12" t="inlineStr">
-        <is>
-          <t>460020450</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="n">
-        <v>7</v>
-      </c>
-      <c r="B13" t="inlineStr"/>
-      <c r="C13" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="D13" t="inlineStr"/>
-      <c r="E13" t="inlineStr">
-        <is>
-          <t>93968775</t>
-        </is>
-      </c>
-      <c r="F13" t="inlineStr">
-        <is>
-          <t>05/29/2026</t>
-        </is>
-      </c>
-      <c r="G13" t="inlineStr">
-        <is>
-          <t>06/08/26</t>
-        </is>
-      </c>
-      <c r="H13" t="inlineStr">
-        <is>
-          <t>NS</t>
-        </is>
-      </c>
-      <c r="I13" t="inlineStr">
-        <is>
-          <t>THE CHARLES MACHINE WORKS Invoice 93968775</t>
-        </is>
-      </c>
-      <c r="J13" t="inlineStr">
-        <is>
-          <t>USD</t>
-        </is>
-      </c>
-      <c r="K13" t="n">
-        <v>212.15</v>
-      </c>
-      <c r="BS13" t="inlineStr"/>
-      <c r="BT13" t="inlineStr">
-        <is>
-          <t>51000100</t>
-        </is>
-      </c>
-      <c r="BU13" t="inlineStr"/>
-      <c r="BV13" t="inlineStr">
-        <is>
-          <t>S</t>
-        </is>
-      </c>
-      <c r="BW13" t="n">
-        <v>212.15</v>
-      </c>
-      <c r="BX13" t="inlineStr">
-        <is>
-          <t>I0</t>
-        </is>
-      </c>
-      <c r="BY13" t="inlineStr"/>
-      <c r="CA13" t="inlineStr">
-        <is>
-          <t>460020450</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="n">
-        <v>8</v>
-      </c>
-      <c r="B14" t="inlineStr"/>
-      <c r="C14" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="D14" t="inlineStr"/>
-      <c r="E14" t="inlineStr">
-        <is>
-          <t>167142</t>
-        </is>
-      </c>
-      <c r="F14" t="inlineStr">
-        <is>
-          <t>01/20/2026</t>
-        </is>
-      </c>
-      <c r="G14" t="inlineStr">
-        <is>
-          <t>06/08/26</t>
-        </is>
-      </c>
-      <c r="H14" t="inlineStr">
-        <is>
-          <t>NS</t>
-        </is>
-      </c>
-      <c r="I14" t="inlineStr">
-        <is>
-          <t>VALVOLINE INSTANT OIL CHANGE Invoice 167142</t>
-        </is>
-      </c>
-      <c r="J14" t="inlineStr">
-        <is>
-          <t>USD</t>
-        </is>
-      </c>
-      <c r="K14" t="n">
-        <v>116.21</v>
-      </c>
-      <c r="BS14" t="inlineStr"/>
-      <c r="BT14" t="inlineStr">
-        <is>
-          <t>51000100</t>
-        </is>
-      </c>
-      <c r="BU14" t="inlineStr"/>
-      <c r="BV14" t="inlineStr">
-        <is>
-          <t>S</t>
-        </is>
-      </c>
-      <c r="BW14" t="n">
-        <v>116.21</v>
-      </c>
-      <c r="BX14" t="inlineStr">
-        <is>
-          <t>I0</t>
-        </is>
-      </c>
-      <c r="BY14" t="inlineStr"/>
-      <c r="CA14" t="inlineStr">
         <is>
           <t>460020450</t>
         </is>

</xml_diff>

<commit_message>
fix 0.1 amount in default
</commit_message>
<xml_diff>
--- a/invoice_automation/clients/northsky_comm/downloads/PROCESSED/invoice_load_001.xlsx
+++ b/invoice_automation/clients/northsky_comm/downloads/PROCESSED/invoice_load_001.xlsx
@@ -580,7 +580,7 @@
     <outlinePr summaryBelow="0"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:DL27"/>
+  <dimension ref="A1:DL48"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.5"/>
   <cols>
     <col width="26" bestFit="1" customWidth="1" style="6" min="1" max="1"/>
@@ -2013,21 +2013,17 @@
           <t>1</t>
         </is>
       </c>
-      <c r="D7" s="23" t="inlineStr">
-        <is>
-          <t>V01732</t>
-        </is>
-      </c>
+      <c r="D7" s="23" t="inlineStr"/>
       <c r="E7" s="23" t="inlineStr">
         <is>
-          <t>UNIVERSAL</t>
+          <t>215749</t>
         </is>
       </c>
       <c r="F7" s="24" t="n">
-        <v>46190</v>
+        <v>46189</v>
       </c>
       <c r="G7" s="24" t="n">
-        <v>46190.67684741095</v>
+        <v>46190.87469867446</v>
       </c>
       <c r="H7" t="inlineStr">
         <is>
@@ -2040,7 +2036,7 @@
         </is>
       </c>
       <c r="K7" s="25" t="n">
-        <v>919.0700000000001</v>
+        <v>1811.43</v>
       </c>
       <c r="BS7" t="n">
         <v>4600</v>
@@ -2061,7 +2057,7 @@
         </is>
       </c>
       <c r="BW7" s="25" t="n">
-        <v>919.0700000000001</v>
+        <v>1811.43</v>
       </c>
       <c r="BX7" t="inlineStr">
         <is>
@@ -2089,19 +2085,19 @@
       </c>
       <c r="D8" s="23" t="inlineStr">
         <is>
-          <t>V02272</t>
+          <t>V02155</t>
         </is>
       </c>
       <c r="E8" s="23" t="inlineStr">
         <is>
-          <t>235377</t>
+          <t>20795</t>
         </is>
       </c>
       <c r="F8" s="24" t="n">
-        <v>46188</v>
+        <v>46189</v>
       </c>
       <c r="G8" s="24" t="n">
-        <v>46190.67684741095</v>
+        <v>46190.87469867446</v>
       </c>
       <c r="H8" t="inlineStr">
         <is>
@@ -2114,7 +2110,7 @@
         </is>
       </c>
       <c r="K8" s="25" t="n">
-        <v>1939.6</v>
+        <v>792.3</v>
       </c>
       <c r="BS8" t="n">
         <v>4600</v>
@@ -2135,7 +2131,7 @@
         </is>
       </c>
       <c r="BW8" s="25" t="n">
-        <v>1939.6</v>
+        <v>792.3</v>
       </c>
       <c r="BX8" t="inlineStr">
         <is>
@@ -2161,21 +2157,17 @@
           <t>1</t>
         </is>
       </c>
-      <c r="D9" s="23" t="inlineStr">
-        <is>
-          <t>V02049</t>
-        </is>
-      </c>
+      <c r="D9" s="23" t="inlineStr"/>
       <c r="E9" s="23" t="inlineStr">
         <is>
-          <t>519156</t>
+          <t>A146008</t>
         </is>
       </c>
       <c r="F9" s="24" t="n">
-        <v>46182</v>
+        <v>46184</v>
       </c>
       <c r="G9" s="24" t="n">
-        <v>46190.67684741095</v>
+        <v>46190.87469868596</v>
       </c>
       <c r="H9" t="inlineStr">
         <is>
@@ -2188,7 +2180,7 @@
         </is>
       </c>
       <c r="K9" s="25" t="n">
-        <v>414.54</v>
+        <v>104.15</v>
       </c>
       <c r="BS9" t="n">
         <v>4600</v>
@@ -2209,7 +2201,7 @@
         </is>
       </c>
       <c r="BW9" s="25" t="n">
-        <v>414.54</v>
+        <v>104.15</v>
       </c>
       <c r="BX9" t="inlineStr">
         <is>
@@ -2235,21 +2227,17 @@
           <t>1</t>
         </is>
       </c>
-      <c r="D10" s="23" t="inlineStr">
-        <is>
-          <t>V01905</t>
-        </is>
-      </c>
+      <c r="D10" s="23" t="inlineStr"/>
       <c r="E10" s="23" t="inlineStr">
         <is>
-          <t>497340</t>
+          <t>17728</t>
         </is>
       </c>
       <c r="F10" s="24" t="n">
-        <v>46189</v>
+        <v>46150</v>
       </c>
       <c r="G10" s="24" t="n">
-        <v>46190.67684742244</v>
+        <v>46190.87469868596</v>
       </c>
       <c r="H10" t="inlineStr">
         <is>
@@ -2262,7 +2250,7 @@
         </is>
       </c>
       <c r="K10" s="25" t="n">
-        <v>217.92</v>
+        <v>922.5</v>
       </c>
       <c r="BS10" t="n">
         <v>4600</v>
@@ -2283,7 +2271,7 @@
         </is>
       </c>
       <c r="BW10" s="25" t="n">
-        <v>217.92</v>
+        <v>922.5</v>
       </c>
       <c r="BX10" t="inlineStr">
         <is>
@@ -2311,19 +2299,19 @@
       </c>
       <c r="D11" s="23" t="inlineStr">
         <is>
-          <t>V01905</t>
+          <t>S00229</t>
         </is>
       </c>
       <c r="E11" s="23" t="inlineStr">
         <is>
-          <t>497344</t>
+          <t>05049629</t>
         </is>
       </c>
       <c r="F11" s="24" t="n">
         <v>46189</v>
       </c>
       <c r="G11" s="24" t="n">
-        <v>46190.67684742244</v>
+        <v>46190.87469868596</v>
       </c>
       <c r="H11" t="inlineStr">
         <is>
@@ -2336,7 +2324,7 @@
         </is>
       </c>
       <c r="K11" s="25" t="n">
-        <v>573.12</v>
+        <v>1607.97</v>
       </c>
       <c r="BS11" t="n">
         <v>4600</v>
@@ -2357,7 +2345,7 @@
         </is>
       </c>
       <c r="BW11" s="25" t="n">
-        <v>573.12</v>
+        <v>1607.97</v>
       </c>
       <c r="BX11" t="inlineStr">
         <is>
@@ -2386,14 +2374,14 @@
       <c r="D12" s="23" t="inlineStr"/>
       <c r="E12" s="23" t="inlineStr">
         <is>
-          <t>2601-143139</t>
+          <t>B13624</t>
         </is>
       </c>
       <c r="F12" s="24" t="n">
         <v>46189</v>
       </c>
       <c r="G12" s="24" t="n">
-        <v>46190.67684742244</v>
+        <v>46190.87469868596</v>
       </c>
       <c r="H12" t="inlineStr">
         <is>
@@ -2406,7 +2394,7 @@
         </is>
       </c>
       <c r="K12" s="25" t="n">
-        <v>55.74</v>
+        <v>218.97</v>
       </c>
       <c r="BS12" t="n">
         <v>4600</v>
@@ -2427,7 +2415,7 @@
         </is>
       </c>
       <c r="BW12" s="25" t="n">
-        <v>55.74</v>
+        <v>218.97</v>
       </c>
       <c r="BX12" t="inlineStr">
         <is>
@@ -2455,19 +2443,19 @@
       </c>
       <c r="D13" s="23" t="inlineStr">
         <is>
-          <t>V01662</t>
+          <t>V01794</t>
         </is>
       </c>
       <c r="E13" s="23" t="inlineStr">
         <is>
-          <t>29253422</t>
+          <t>190359</t>
         </is>
       </c>
       <c r="F13" s="24" t="n">
         <v>46189</v>
       </c>
       <c r="G13" s="24" t="n">
-        <v>46190.67684742244</v>
+        <v>46190.87469868596</v>
       </c>
       <c r="H13" t="inlineStr">
         <is>
@@ -2480,7 +2468,7 @@
         </is>
       </c>
       <c r="K13" s="25" t="n">
-        <v>73.16</v>
+        <v>1120</v>
       </c>
       <c r="BS13" t="n">
         <v>4600</v>
@@ -2501,7 +2489,7 @@
         </is>
       </c>
       <c r="BW13" s="25" t="n">
-        <v>73.16</v>
+        <v>1120</v>
       </c>
       <c r="BX13" t="inlineStr">
         <is>
@@ -2527,21 +2515,17 @@
           <t>1</t>
         </is>
       </c>
-      <c r="D14" s="23" t="inlineStr">
-        <is>
-          <t>V01662</t>
-        </is>
-      </c>
+      <c r="D14" s="23" t="inlineStr"/>
       <c r="E14" s="23" t="inlineStr">
         <is>
-          <t>30238729</t>
+          <t>3213755</t>
         </is>
       </c>
       <c r="F14" s="24" t="n">
-        <v>46189</v>
+        <v>46156</v>
       </c>
       <c r="G14" s="24" t="n">
-        <v>46190.67684742244</v>
+        <v>46190.8746986981</v>
       </c>
       <c r="H14" t="inlineStr">
         <is>
@@ -2554,7 +2538,7 @@
         </is>
       </c>
       <c r="K14" s="25" t="n">
-        <v>9.99</v>
+        <v>165.6</v>
       </c>
       <c r="BS14" t="n">
         <v>4600</v>
@@ -2575,7 +2559,7 @@
         </is>
       </c>
       <c r="BW14" s="25" t="n">
-        <v>9.99</v>
+        <v>165.6</v>
       </c>
       <c r="BX14" t="inlineStr">
         <is>
@@ -2603,19 +2587,19 @@
       </c>
       <c r="D15" s="23" t="inlineStr">
         <is>
-          <t>V01476</t>
+          <t>V02000</t>
         </is>
       </c>
       <c r="E15" s="23" t="inlineStr">
         <is>
-          <t>9954158524</t>
+          <t>120376-01</t>
         </is>
       </c>
       <c r="F15" s="24" t="n">
         <v>46189</v>
       </c>
       <c r="G15" s="24" t="n">
-        <v>46190.67684742244</v>
+        <v>46190.8746986981</v>
       </c>
       <c r="H15" t="inlineStr">
         <is>
@@ -2628,7 +2612,7 @@
         </is>
       </c>
       <c r="K15" s="25" t="n">
-        <v>276.34</v>
+        <v>1234.8</v>
       </c>
       <c r="BS15" t="n">
         <v>4600</v>
@@ -2649,7 +2633,7 @@
         </is>
       </c>
       <c r="BW15" s="25" t="n">
-        <v>276.34</v>
+        <v>1234.8</v>
       </c>
       <c r="BX15" t="inlineStr">
         <is>
@@ -2677,19 +2661,19 @@
       </c>
       <c r="D16" s="23" t="inlineStr">
         <is>
-          <t>V01667</t>
+          <t>V01904</t>
         </is>
       </c>
       <c r="E16" s="23" t="inlineStr">
         <is>
-          <t>3233785</t>
+          <t>ENGINEERING</t>
         </is>
       </c>
       <c r="F16" s="24" t="n">
-        <v>46183</v>
+        <v>46189</v>
       </c>
       <c r="G16" s="24" t="n">
-        <v>46190.67684742244</v>
+        <v>46190.8746986981</v>
       </c>
       <c r="H16" t="inlineStr">
         <is>
@@ -2702,7 +2686,7 @@
         </is>
       </c>
       <c r="K16" s="25" t="n">
-        <v>488</v>
+        <v>1050</v>
       </c>
       <c r="BS16" t="n">
         <v>4600</v>
@@ -2723,7 +2707,7 @@
         </is>
       </c>
       <c r="BW16" s="25" t="n">
-        <v>488</v>
+        <v>1050</v>
       </c>
       <c r="BX16" t="inlineStr">
         <is>
@@ -2751,19 +2735,19 @@
       </c>
       <c r="D17" s="23" t="inlineStr">
         <is>
-          <t>S00593</t>
+          <t>V08720</t>
         </is>
       </c>
       <c r="E17" s="23" t="inlineStr">
         <is>
-          <t>513329</t>
+          <t>11419</t>
         </is>
       </c>
       <c r="F17" s="24" t="n">
         <v>46189</v>
       </c>
       <c r="G17" s="24" t="n">
-        <v>46190.67684742244</v>
+        <v>46190.8746986981</v>
       </c>
       <c r="H17" t="inlineStr">
         <is>
@@ -2776,7 +2760,7 @@
         </is>
       </c>
       <c r="K17" s="25" t="n">
-        <v>129.86</v>
+        <v>11909.02</v>
       </c>
       <c r="BS17" t="n">
         <v>4600</v>
@@ -2797,7 +2781,7 @@
         </is>
       </c>
       <c r="BW17" s="25" t="n">
-        <v>129.86</v>
+        <v>11909.02</v>
       </c>
       <c r="BX17" t="inlineStr">
         <is>
@@ -2825,19 +2809,19 @@
       </c>
       <c r="D18" s="23" t="inlineStr">
         <is>
-          <t>V01669</t>
+          <t>V08720</t>
         </is>
       </c>
       <c r="E18" s="23" t="inlineStr">
         <is>
-          <t>134937</t>
+          <t>11420</t>
         </is>
       </c>
       <c r="F18" s="24" t="n">
-        <v>46181</v>
+        <v>46189</v>
       </c>
       <c r="G18" s="24" t="n">
-        <v>46190.67684742244</v>
+        <v>46190.8746986981</v>
       </c>
       <c r="H18" t="inlineStr">
         <is>
@@ -2850,7 +2834,7 @@
         </is>
       </c>
       <c r="K18" s="25" t="n">
-        <v>990</v>
+        <v>1182.31</v>
       </c>
       <c r="BS18" t="n">
         <v>4600</v>
@@ -2871,7 +2855,7 @@
         </is>
       </c>
       <c r="BW18" s="25" t="n">
-        <v>990</v>
+        <v>1182.31</v>
       </c>
       <c r="BX18" t="inlineStr">
         <is>
@@ -2899,19 +2883,19 @@
       </c>
       <c r="D19" s="23" t="inlineStr">
         <is>
-          <t>V01830</t>
+          <t>V02209</t>
         </is>
       </c>
       <c r="E19" s="23" t="inlineStr">
         <is>
-          <t>CD99330352</t>
+          <t>30004348</t>
         </is>
       </c>
       <c r="F19" s="24" t="n">
-        <v>46184</v>
+        <v>46156</v>
       </c>
       <c r="G19" s="24" t="n">
-        <v>46190.67684742244</v>
+        <v>46190.8746986981</v>
       </c>
       <c r="H19" t="inlineStr">
         <is>
@@ -2924,7 +2908,7 @@
         </is>
       </c>
       <c r="K19" s="25" t="n">
-        <v>1652</v>
+        <v>525.22</v>
       </c>
       <c r="BS19" t="n">
         <v>4600</v>
@@ -2945,7 +2929,7 @@
         </is>
       </c>
       <c r="BW19" s="25" t="n">
-        <v>1652</v>
+        <v>525.22</v>
       </c>
       <c r="BX19" t="inlineStr">
         <is>
@@ -2973,19 +2957,19 @@
       </c>
       <c r="D20" s="23" t="inlineStr">
         <is>
-          <t>V02253</t>
+          <t>V02240</t>
         </is>
       </c>
       <c r="E20" s="23" t="inlineStr">
         <is>
-          <t>654643</t>
+          <t>51486</t>
         </is>
       </c>
       <c r="F20" s="24" t="n">
-        <v>46189</v>
+        <v>46183</v>
       </c>
       <c r="G20" s="24" t="n">
-        <v>46190.67684742244</v>
+        <v>46190.87469870926</v>
       </c>
       <c r="H20" t="inlineStr">
         <is>
@@ -2998,7 +2982,7 @@
         </is>
       </c>
       <c r="K20" s="25" t="n">
-        <v>100</v>
+        <v>90</v>
       </c>
       <c r="BS20" t="n">
         <v>4600</v>
@@ -3019,7 +3003,7 @@
         </is>
       </c>
       <c r="BW20" s="25" t="n">
-        <v>100</v>
+        <v>90</v>
       </c>
       <c r="BX20" t="inlineStr">
         <is>
@@ -3047,19 +3031,19 @@
       </c>
       <c r="D21" s="23" t="inlineStr">
         <is>
-          <t>S00863</t>
+          <t>V04626</t>
         </is>
       </c>
       <c r="E21" s="23" t="inlineStr">
         <is>
-          <t>14315</t>
+          <t>100401270</t>
         </is>
       </c>
       <c r="F21" s="24" t="n">
-        <v>46189</v>
+        <v>46184</v>
       </c>
       <c r="G21" s="24" t="n">
-        <v>46190.67684742244</v>
+        <v>46190.87469872115</v>
       </c>
       <c r="H21" t="inlineStr">
         <is>
@@ -3072,7 +3056,7 @@
         </is>
       </c>
       <c r="K21" s="25" t="n">
-        <v>1650</v>
+        <v>53723512</v>
       </c>
       <c r="BS21" t="n">
         <v>4600</v>
@@ -3093,7 +3077,7 @@
         </is>
       </c>
       <c r="BW21" s="25" t="n">
-        <v>1650</v>
+        <v>53723512</v>
       </c>
       <c r="BX21" t="inlineStr">
         <is>
@@ -3121,19 +3105,19 @@
       </c>
       <c r="D22" s="23" t="inlineStr">
         <is>
-          <t>V01737</t>
+          <t>V02261</t>
         </is>
       </c>
       <c r="E22" s="23" t="inlineStr">
         <is>
-          <t>SI-81478</t>
+          <t>202606-423</t>
         </is>
       </c>
       <c r="F22" s="24" t="n">
-        <v>46185</v>
+        <v>46189</v>
       </c>
       <c r="G22" s="24" t="n">
-        <v>46190.67684743405</v>
+        <v>46190.87469872115</v>
       </c>
       <c r="H22" t="inlineStr">
         <is>
@@ -3146,7 +3130,7 @@
         </is>
       </c>
       <c r="K22" s="25" t="n">
-        <v>72.83</v>
+        <v>100</v>
       </c>
       <c r="BS22" t="n">
         <v>4600</v>
@@ -3167,7 +3151,7 @@
         </is>
       </c>
       <c r="BW22" s="25" t="n">
-        <v>72.83</v>
+        <v>100</v>
       </c>
       <c r="BX22" t="inlineStr">
         <is>
@@ -3195,19 +3179,19 @@
       </c>
       <c r="D23" s="23" t="inlineStr">
         <is>
-          <t>V00052</t>
+          <t>V04811</t>
         </is>
       </c>
       <c r="E23" s="23" t="inlineStr">
         <is>
-          <t>176297598-0009</t>
+          <t>CONSTRUCTION</t>
         </is>
       </c>
       <c r="F23" s="24" t="n">
-        <v>46186</v>
+        <v>46189</v>
       </c>
       <c r="G23" s="24" t="n">
-        <v>46190.67684743405</v>
+        <v>46190.87469872115</v>
       </c>
       <c r="H23" t="inlineStr">
         <is>
@@ -3220,7 +3204,7 @@
         </is>
       </c>
       <c r="K23" s="25" t="n">
-        <v>2397.26</v>
+        <v>782.27</v>
       </c>
       <c r="BS23" t="n">
         <v>4600</v>
@@ -3241,7 +3225,7 @@
         </is>
       </c>
       <c r="BW23" s="25" t="n">
-        <v>2397.26</v>
+        <v>782.27</v>
       </c>
       <c r="BX23" t="inlineStr">
         <is>
@@ -3269,19 +3253,19 @@
       </c>
       <c r="D24" s="23" t="inlineStr">
         <is>
-          <t>V01649</t>
+          <t>V04811</t>
         </is>
       </c>
       <c r="E24" s="23" t="inlineStr">
         <is>
-          <t>261780918-002</t>
+          <t>CONTRUCTION</t>
         </is>
       </c>
       <c r="F24" s="24" t="n">
-        <v>46185</v>
+        <v>46189</v>
       </c>
       <c r="G24" s="24" t="n">
-        <v>46190.67684743405</v>
+        <v>46190.87469872115</v>
       </c>
       <c r="H24" t="inlineStr">
         <is>
@@ -3294,7 +3278,7 @@
         </is>
       </c>
       <c r="K24" s="25" t="n">
-        <v>1488.69</v>
+        <v>114.75</v>
       </c>
       <c r="BS24" t="n">
         <v>4600</v>
@@ -3315,7 +3299,7 @@
         </is>
       </c>
       <c r="BW24" s="25" t="n">
-        <v>1488.69</v>
+        <v>114.75</v>
       </c>
       <c r="BX24" t="inlineStr">
         <is>
@@ -3343,19 +3327,19 @@
       </c>
       <c r="D25" s="23" t="inlineStr">
         <is>
-          <t>V01651</t>
+          <t>V02275</t>
         </is>
       </c>
       <c r="E25" s="23" t="inlineStr">
         <is>
-          <t>6688591</t>
+          <t>120336</t>
         </is>
       </c>
       <c r="F25" s="24" t="n">
-        <v>46185</v>
+        <v>46143</v>
       </c>
       <c r="G25" s="24" t="n">
-        <v>46190.67684743405</v>
+        <v>46190.87469872115</v>
       </c>
       <c r="H25" t="inlineStr">
         <is>
@@ -3368,7 +3352,7 @@
         </is>
       </c>
       <c r="K25" s="25" t="n">
-        <v>1941.12</v>
+        <v>310</v>
       </c>
       <c r="BS25" t="n">
         <v>4600</v>
@@ -3389,7 +3373,7 @@
         </is>
       </c>
       <c r="BW25" s="25" t="n">
-        <v>1941.12</v>
+        <v>310</v>
       </c>
       <c r="BX25" t="inlineStr">
         <is>
@@ -3417,19 +3401,19 @@
       </c>
       <c r="D26" s="23" t="inlineStr">
         <is>
-          <t>V05171</t>
+          <t>V02275</t>
         </is>
       </c>
       <c r="E26" s="23" t="inlineStr">
         <is>
-          <t>S100252088.001</t>
+          <t>120716</t>
         </is>
       </c>
       <c r="F26" s="24" t="n">
-        <v>46188</v>
+        <v>46174</v>
       </c>
       <c r="G26" s="24" t="n">
-        <v>46190.67684743405</v>
+        <v>46190.87469873242</v>
       </c>
       <c r="H26" t="inlineStr">
         <is>
@@ -3442,7 +3426,7 @@
         </is>
       </c>
       <c r="K26" s="25" t="n">
-        <v>291.59</v>
+        <v>310</v>
       </c>
       <c r="BS26" t="n">
         <v>4600</v>
@@ -3463,7 +3447,7 @@
         </is>
       </c>
       <c r="BW26" s="25" t="n">
-        <v>291.59</v>
+        <v>310</v>
       </c>
       <c r="BX26" t="inlineStr">
         <is>
@@ -3491,19 +3475,19 @@
       </c>
       <c r="D27" s="23" t="inlineStr">
         <is>
-          <t>V00033</t>
+          <t>V02253</t>
         </is>
       </c>
       <c r="E27" s="23" t="inlineStr">
         <is>
-          <t>10023216691</t>
+          <t>654643</t>
         </is>
       </c>
       <c r="F27" s="24" t="n">
-        <v>46083</v>
+        <v>46189</v>
       </c>
       <c r="G27" s="24" t="n">
-        <v>46190.67684743405</v>
+        <v>46190.87469873242</v>
       </c>
       <c r="H27" t="inlineStr">
         <is>
@@ -3516,7 +3500,7 @@
         </is>
       </c>
       <c r="K27" s="25" t="n">
-        <v>793.76</v>
+        <v>100</v>
       </c>
       <c r="BS27" t="n">
         <v>4600</v>
@@ -3528,7 +3512,7 @@
       </c>
       <c r="BU27" s="23" t="inlineStr">
         <is>
-          <t>suppllies</t>
+          <t>Supplies</t>
         </is>
       </c>
       <c r="BV27" t="inlineStr">
@@ -3537,7 +3521,7 @@
         </is>
       </c>
       <c r="BW27" s="25" t="n">
-        <v>793.76</v>
+        <v>100</v>
       </c>
       <c r="BX27" t="inlineStr">
         <is>
@@ -3546,6 +3530,1540 @@
       </c>
       <c r="BY27" t="inlineStr"/>
       <c r="CA27" t="inlineStr">
+        <is>
+          <t>460020450</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="n">
+        <v>22</v>
+      </c>
+      <c r="B28" t="n">
+        <v>4600</v>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D28" s="23" t="inlineStr"/>
+      <c r="E28" s="23" t="inlineStr">
+        <is>
+          <t>50010</t>
+        </is>
+      </c>
+      <c r="F28" s="24" t="n">
+        <v>46189</v>
+      </c>
+      <c r="G28" s="24" t="n">
+        <v>46190.87469873242</v>
+      </c>
+      <c r="H28" t="inlineStr">
+        <is>
+          <t>NS</t>
+        </is>
+      </c>
+      <c r="J28" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="K28" s="25" t="n">
+        <v>100</v>
+      </c>
+      <c r="BS28" t="n">
+        <v>4600</v>
+      </c>
+      <c r="BT28" t="inlineStr">
+        <is>
+          <t>51000100</t>
+        </is>
+      </c>
+      <c r="BU28" s="23" t="inlineStr">
+        <is>
+          <t>Supplies</t>
+        </is>
+      </c>
+      <c r="BV28" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="BW28" s="25" t="n">
+        <v>100</v>
+      </c>
+      <c r="BX28" t="inlineStr">
+        <is>
+          <t>I0</t>
+        </is>
+      </c>
+      <c r="BY28" t="inlineStr"/>
+      <c r="CA28" t="inlineStr">
+        <is>
+          <t>460020450</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="n">
+        <v>23</v>
+      </c>
+      <c r="B29" t="n">
+        <v>4600</v>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D29" s="23" t="inlineStr">
+        <is>
+          <t>S00863</t>
+        </is>
+      </c>
+      <c r="E29" s="23" t="inlineStr">
+        <is>
+          <t>14315</t>
+        </is>
+      </c>
+      <c r="F29" s="24" t="n">
+        <v>46189</v>
+      </c>
+      <c r="G29" s="24" t="n">
+        <v>46190.87469873242</v>
+      </c>
+      <c r="H29" t="inlineStr">
+        <is>
+          <t>NS</t>
+        </is>
+      </c>
+      <c r="J29" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="K29" s="25" t="n">
+        <v>1650</v>
+      </c>
+      <c r="BS29" t="n">
+        <v>4600</v>
+      </c>
+      <c r="BT29" t="inlineStr">
+        <is>
+          <t>51000100</t>
+        </is>
+      </c>
+      <c r="BU29" s="23" t="inlineStr">
+        <is>
+          <t>Supplies</t>
+        </is>
+      </c>
+      <c r="BV29" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="BW29" s="25" t="n">
+        <v>1650</v>
+      </c>
+      <c r="BX29" t="inlineStr">
+        <is>
+          <t>I0</t>
+        </is>
+      </c>
+      <c r="BY29" t="inlineStr"/>
+      <c r="CA29" t="inlineStr">
+        <is>
+          <t>460020450</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="n">
+        <v>24</v>
+      </c>
+      <c r="B30" t="n">
+        <v>4600</v>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D30" s="23" t="inlineStr">
+        <is>
+          <t>S00278</t>
+        </is>
+      </c>
+      <c r="E30" s="23" t="inlineStr">
+        <is>
+          <t>12386</t>
+        </is>
+      </c>
+      <c r="F30" s="24" t="n">
+        <v>46134</v>
+      </c>
+      <c r="G30" s="24" t="n">
+        <v>46190.87469873242</v>
+      </c>
+      <c r="H30" t="inlineStr">
+        <is>
+          <t>NS</t>
+        </is>
+      </c>
+      <c r="J30" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="K30" s="25" t="n">
+        <v>336.5</v>
+      </c>
+      <c r="BS30" t="n">
+        <v>4600</v>
+      </c>
+      <c r="BT30" t="inlineStr">
+        <is>
+          <t>51000100</t>
+        </is>
+      </c>
+      <c r="BU30" s="23" t="inlineStr">
+        <is>
+          <t>Supplies</t>
+        </is>
+      </c>
+      <c r="BV30" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="BW30" s="25" t="n">
+        <v>336.5</v>
+      </c>
+      <c r="BX30" t="inlineStr">
+        <is>
+          <t>I0</t>
+        </is>
+      </c>
+      <c r="BY30" t="inlineStr"/>
+      <c r="CA30" t="inlineStr">
+        <is>
+          <t>460020450</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="n">
+        <v>25</v>
+      </c>
+      <c r="B31" t="n">
+        <v>4600</v>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D31" s="23" t="inlineStr">
+        <is>
+          <t>V04110</t>
+        </is>
+      </c>
+      <c r="E31" s="23" t="inlineStr">
+        <is>
+          <t>12394</t>
+        </is>
+      </c>
+      <c r="F31" s="24" t="n">
+        <v>46141</v>
+      </c>
+      <c r="G31" s="24" t="n">
+        <v>46190.87469873242</v>
+      </c>
+      <c r="H31" t="inlineStr">
+        <is>
+          <t>NS</t>
+        </is>
+      </c>
+      <c r="J31" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="K31" s="25" t="n">
+        <v>1199.34</v>
+      </c>
+      <c r="BS31" t="n">
+        <v>4600</v>
+      </c>
+      <c r="BT31" t="inlineStr">
+        <is>
+          <t>51000100</t>
+        </is>
+      </c>
+      <c r="BU31" s="23" t="inlineStr">
+        <is>
+          <t>Supplies</t>
+        </is>
+      </c>
+      <c r="BV31" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="BW31" s="25" t="n">
+        <v>1199.34</v>
+      </c>
+      <c r="BX31" t="inlineStr">
+        <is>
+          <t>I0</t>
+        </is>
+      </c>
+      <c r="BY31" t="inlineStr"/>
+      <c r="CA31" t="inlineStr">
+        <is>
+          <t>460020450</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="n">
+        <v>26</v>
+      </c>
+      <c r="B32" t="n">
+        <v>4600</v>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D32" s="23" t="inlineStr">
+        <is>
+          <t>V03648</t>
+        </is>
+      </c>
+      <c r="E32" s="23" t="inlineStr">
+        <is>
+          <t>122865</t>
+        </is>
+      </c>
+      <c r="F32" s="24" t="n">
+        <v>46189</v>
+      </c>
+      <c r="G32" s="24" t="n">
+        <v>46190.8746987439</v>
+      </c>
+      <c r="H32" t="inlineStr">
+        <is>
+          <t>NS</t>
+        </is>
+      </c>
+      <c r="J32" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="K32" s="25" t="n">
+        <v>215.5</v>
+      </c>
+      <c r="BS32" t="n">
+        <v>4600</v>
+      </c>
+      <c r="BT32" t="inlineStr">
+        <is>
+          <t>51000100</t>
+        </is>
+      </c>
+      <c r="BU32" s="23" t="inlineStr">
+        <is>
+          <t>Supplies</t>
+        </is>
+      </c>
+      <c r="BV32" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="BW32" s="25" t="n">
+        <v>215.5</v>
+      </c>
+      <c r="BX32" t="inlineStr">
+        <is>
+          <t>I0</t>
+        </is>
+      </c>
+      <c r="BY32" t="inlineStr"/>
+      <c r="CA32" t="inlineStr">
+        <is>
+          <t>460020450</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="n">
+        <v>27</v>
+      </c>
+      <c r="B33" t="n">
+        <v>4600</v>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D33" s="23" t="inlineStr">
+        <is>
+          <t>V02283</t>
+        </is>
+      </c>
+      <c r="E33" s="23" t="inlineStr">
+        <is>
+          <t>SUPPLY</t>
+        </is>
+      </c>
+      <c r="F33" s="24" t="n">
+        <v>45847</v>
+      </c>
+      <c r="G33" s="24" t="n">
+        <v>46190.8746987439</v>
+      </c>
+      <c r="H33" t="inlineStr">
+        <is>
+          <t>NS</t>
+        </is>
+      </c>
+      <c r="J33" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="K33" s="25" t="n">
+        <v>19.57</v>
+      </c>
+      <c r="BS33" t="n">
+        <v>4600</v>
+      </c>
+      <c r="BT33" t="inlineStr">
+        <is>
+          <t>51000100</t>
+        </is>
+      </c>
+      <c r="BU33" s="23" t="inlineStr">
+        <is>
+          <t>Supplies</t>
+        </is>
+      </c>
+      <c r="BV33" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="BW33" s="25" t="n">
+        <v>19.57</v>
+      </c>
+      <c r="BX33" t="inlineStr">
+        <is>
+          <t>I0</t>
+        </is>
+      </c>
+      <c r="BY33" t="inlineStr"/>
+      <c r="CA33" t="inlineStr">
+        <is>
+          <t>460020450</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="n">
+        <v>28</v>
+      </c>
+      <c r="B34" t="n">
+        <v>4600</v>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D34" s="23" t="inlineStr"/>
+      <c r="E34" s="23" t="inlineStr">
+        <is>
+          <t>268325</t>
+        </is>
+      </c>
+      <c r="F34" s="24" t="n">
+        <v>46189</v>
+      </c>
+      <c r="G34" s="24" t="n">
+        <v>46190.8746987439</v>
+      </c>
+      <c r="H34" t="inlineStr">
+        <is>
+          <t>NS</t>
+        </is>
+      </c>
+      <c r="J34" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="K34" s="25" t="n">
+        <v>971.05</v>
+      </c>
+      <c r="BS34" t="n">
+        <v>4600</v>
+      </c>
+      <c r="BT34" t="inlineStr">
+        <is>
+          <t>51000100</t>
+        </is>
+      </c>
+      <c r="BU34" s="23" t="inlineStr">
+        <is>
+          <t>Supplies</t>
+        </is>
+      </c>
+      <c r="BV34" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="BW34" s="25" t="n">
+        <v>971.05</v>
+      </c>
+      <c r="BX34" t="inlineStr">
+        <is>
+          <t>I0</t>
+        </is>
+      </c>
+      <c r="BY34" t="inlineStr"/>
+      <c r="CA34" t="inlineStr">
+        <is>
+          <t>460020450</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="n">
+        <v>29</v>
+      </c>
+      <c r="B35" t="n">
+        <v>4600</v>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D35" s="23" t="inlineStr"/>
+      <c r="E35" s="23" t="inlineStr">
+        <is>
+          <t>268413</t>
+        </is>
+      </c>
+      <c r="F35" s="24" t="n">
+        <v>46189</v>
+      </c>
+      <c r="G35" s="24" t="n">
+        <v>46190.8746987439</v>
+      </c>
+      <c r="H35" t="inlineStr">
+        <is>
+          <t>NS</t>
+        </is>
+      </c>
+      <c r="J35" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="K35" s="25" t="n">
+        <v>24.26</v>
+      </c>
+      <c r="BS35" t="n">
+        <v>4600</v>
+      </c>
+      <c r="BT35" t="inlineStr">
+        <is>
+          <t>51000100</t>
+        </is>
+      </c>
+      <c r="BU35" s="23" t="inlineStr">
+        <is>
+          <t>Supplies</t>
+        </is>
+      </c>
+      <c r="BV35" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="BW35" s="25" t="n">
+        <v>24.26</v>
+      </c>
+      <c r="BX35" t="inlineStr">
+        <is>
+          <t>I0</t>
+        </is>
+      </c>
+      <c r="BY35" t="inlineStr"/>
+      <c r="CA35" t="inlineStr">
+        <is>
+          <t>460020450</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="n">
+        <v>30</v>
+      </c>
+      <c r="B36" t="n">
+        <v>4600</v>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D36" s="23" t="inlineStr">
+        <is>
+          <t>V02289</t>
+        </is>
+      </c>
+      <c r="E36" s="23" t="inlineStr">
+        <is>
+          <t>INV0067435</t>
+        </is>
+      </c>
+      <c r="F36" s="24" t="n">
+        <v>46171</v>
+      </c>
+      <c r="G36" s="24" t="n">
+        <v>46190.8746987439</v>
+      </c>
+      <c r="H36" t="inlineStr">
+        <is>
+          <t>NS</t>
+        </is>
+      </c>
+      <c r="J36" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="K36" s="25" t="n">
+        <v>511.13</v>
+      </c>
+      <c r="BS36" t="n">
+        <v>4600</v>
+      </c>
+      <c r="BT36" t="inlineStr">
+        <is>
+          <t>51000100</t>
+        </is>
+      </c>
+      <c r="BU36" s="23" t="inlineStr">
+        <is>
+          <t>Supplies</t>
+        </is>
+      </c>
+      <c r="BV36" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="BW36" s="25" t="n">
+        <v>511.13</v>
+      </c>
+      <c r="BX36" t="inlineStr">
+        <is>
+          <t>I0</t>
+        </is>
+      </c>
+      <c r="BY36" t="inlineStr"/>
+      <c r="CA36" t="inlineStr">
+        <is>
+          <t>460020450</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="n">
+        <v>31</v>
+      </c>
+      <c r="B37" t="n">
+        <v>4600</v>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D37" s="23" t="inlineStr">
+        <is>
+          <t>V03684</t>
+        </is>
+      </c>
+      <c r="E37" s="23" t="inlineStr">
+        <is>
+          <t>IN-159430</t>
+        </is>
+      </c>
+      <c r="F37" s="24" t="n">
+        <v>46120</v>
+      </c>
+      <c r="G37" s="24" t="n">
+        <v>46190.8746987439</v>
+      </c>
+      <c r="H37" t="inlineStr">
+        <is>
+          <t>NS</t>
+        </is>
+      </c>
+      <c r="J37" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="K37" s="25" t="n">
+        <v>181.25</v>
+      </c>
+      <c r="BS37" t="n">
+        <v>4600</v>
+      </c>
+      <c r="BT37" t="inlineStr">
+        <is>
+          <t>51000100</t>
+        </is>
+      </c>
+      <c r="BU37" s="23" t="inlineStr">
+        <is>
+          <t>Supplies</t>
+        </is>
+      </c>
+      <c r="BV37" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="BW37" s="25" t="n">
+        <v>181.25</v>
+      </c>
+      <c r="BX37" t="inlineStr">
+        <is>
+          <t>I0</t>
+        </is>
+      </c>
+      <c r="BY37" t="inlineStr"/>
+      <c r="CA37" t="inlineStr">
+        <is>
+          <t>460020450</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="n">
+        <v>32</v>
+      </c>
+      <c r="B38" t="n">
+        <v>4600</v>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D38" s="23" t="inlineStr">
+        <is>
+          <t>V01613</t>
+        </is>
+      </c>
+      <c r="E38" s="23" t="inlineStr">
+        <is>
+          <t>273647</t>
+        </is>
+      </c>
+      <c r="F38" s="24" t="n">
+        <v>46189</v>
+      </c>
+      <c r="G38" s="24" t="n">
+        <v>46190.87469875543</v>
+      </c>
+      <c r="H38" t="inlineStr">
+        <is>
+          <t>NS</t>
+        </is>
+      </c>
+      <c r="J38" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="K38" s="25" t="n">
+        <v>225</v>
+      </c>
+      <c r="BS38" t="n">
+        <v>4600</v>
+      </c>
+      <c r="BT38" t="inlineStr">
+        <is>
+          <t>51000100</t>
+        </is>
+      </c>
+      <c r="BU38" s="23" t="inlineStr">
+        <is>
+          <t>Supplies</t>
+        </is>
+      </c>
+      <c r="BV38" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="BW38" s="25" t="n">
+        <v>225</v>
+      </c>
+      <c r="BX38" t="inlineStr">
+        <is>
+          <t>I0</t>
+        </is>
+      </c>
+      <c r="BY38" t="inlineStr"/>
+      <c r="CA38" t="inlineStr">
+        <is>
+          <t>460020450</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="n">
+        <v>33</v>
+      </c>
+      <c r="B39" t="n">
+        <v>4600</v>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D39" s="23" t="inlineStr"/>
+      <c r="E39" s="23" t="inlineStr">
+        <is>
+          <t>1597060126</t>
+        </is>
+      </c>
+      <c r="F39" s="24" t="n">
+        <v>46189</v>
+      </c>
+      <c r="G39" s="24" t="n">
+        <v>46190.87469875543</v>
+      </c>
+      <c r="H39" t="inlineStr">
+        <is>
+          <t>NS</t>
+        </is>
+      </c>
+      <c r="J39" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="K39" s="25" t="n">
+        <v>150</v>
+      </c>
+      <c r="BS39" t="n">
+        <v>4600</v>
+      </c>
+      <c r="BT39" t="inlineStr">
+        <is>
+          <t>51000100</t>
+        </is>
+      </c>
+      <c r="BU39" s="23" t="inlineStr">
+        <is>
+          <t>Supplies</t>
+        </is>
+      </c>
+      <c r="BV39" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="BW39" s="25" t="n">
+        <v>150</v>
+      </c>
+      <c r="BX39" t="inlineStr">
+        <is>
+          <t>I0</t>
+        </is>
+      </c>
+      <c r="BY39" t="inlineStr"/>
+      <c r="CA39" t="inlineStr">
+        <is>
+          <t>460020450</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="n">
+        <v>34</v>
+      </c>
+      <c r="B40" t="n">
+        <v>4600</v>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D40" s="23" t="inlineStr">
+        <is>
+          <t>V01818</t>
+        </is>
+      </c>
+      <c r="E40" s="23" t="inlineStr">
+        <is>
+          <t>00105333</t>
+        </is>
+      </c>
+      <c r="F40" s="24" t="n">
+        <v>46137</v>
+      </c>
+      <c r="G40" s="24" t="n">
+        <v>46190.87469875543</v>
+      </c>
+      <c r="H40" t="inlineStr">
+        <is>
+          <t>NS</t>
+        </is>
+      </c>
+      <c r="J40" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="K40" s="25" t="n">
+        <v>1035</v>
+      </c>
+      <c r="BS40" t="n">
+        <v>4600</v>
+      </c>
+      <c r="BT40" t="inlineStr">
+        <is>
+          <t>51000100</t>
+        </is>
+      </c>
+      <c r="BU40" s="23" t="inlineStr">
+        <is>
+          <t>Supplies</t>
+        </is>
+      </c>
+      <c r="BV40" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="BW40" s="25" t="n">
+        <v>1035</v>
+      </c>
+      <c r="BX40" t="inlineStr">
+        <is>
+          <t>I0</t>
+        </is>
+      </c>
+      <c r="BY40" t="inlineStr"/>
+      <c r="CA40" t="inlineStr">
+        <is>
+          <t>460020450</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="n">
+        <v>35</v>
+      </c>
+      <c r="B41" t="n">
+        <v>4600</v>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D41" s="23" t="inlineStr"/>
+      <c r="E41" s="23" t="inlineStr">
+        <is>
+          <t>18771</t>
+        </is>
+      </c>
+      <c r="F41" s="24" t="n">
+        <v>46189</v>
+      </c>
+      <c r="G41" s="24" t="n">
+        <v>46190.87469875543</v>
+      </c>
+      <c r="H41" t="inlineStr">
+        <is>
+          <t>NS</t>
+        </is>
+      </c>
+      <c r="J41" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="K41" s="25" t="n">
+        <v>1096.27</v>
+      </c>
+      <c r="BS41" t="n">
+        <v>4600</v>
+      </c>
+      <c r="BT41" t="inlineStr">
+        <is>
+          <t>51000100</t>
+        </is>
+      </c>
+      <c r="BU41" s="23" t="inlineStr">
+        <is>
+          <t>Supplies</t>
+        </is>
+      </c>
+      <c r="BV41" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="BW41" s="25" t="n">
+        <v>1096.27</v>
+      </c>
+      <c r="BX41" t="inlineStr">
+        <is>
+          <t>I0</t>
+        </is>
+      </c>
+      <c r="BY41" t="inlineStr"/>
+      <c r="CA41" t="inlineStr">
+        <is>
+          <t>460020450</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="n">
+        <v>36</v>
+      </c>
+      <c r="B42" t="n">
+        <v>4600</v>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D42" s="23" t="inlineStr">
+        <is>
+          <t>S00498</t>
+        </is>
+      </c>
+      <c r="E42" s="23" t="inlineStr">
+        <is>
+          <t>CONTROL</t>
+        </is>
+      </c>
+      <c r="F42" s="24" t="n">
+        <v>46189</v>
+      </c>
+      <c r="G42" s="24" t="n">
+        <v>46190.87469875543</v>
+      </c>
+      <c r="H42" t="inlineStr">
+        <is>
+          <t>NS</t>
+        </is>
+      </c>
+      <c r="J42" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="K42" s="25" t="n">
+        <v>6</v>
+      </c>
+      <c r="BS42" t="n">
+        <v>4600</v>
+      </c>
+      <c r="BT42" t="inlineStr">
+        <is>
+          <t>51000100</t>
+        </is>
+      </c>
+      <c r="BU42" s="23" t="inlineStr">
+        <is>
+          <t>Supplies</t>
+        </is>
+      </c>
+      <c r="BV42" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="BW42" s="25" t="n">
+        <v>6</v>
+      </c>
+      <c r="BX42" t="inlineStr">
+        <is>
+          <t>I0</t>
+        </is>
+      </c>
+      <c r="BY42" t="inlineStr"/>
+      <c r="CA42" t="inlineStr">
+        <is>
+          <t>460020450</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="n">
+        <v>37</v>
+      </c>
+      <c r="B43" t="n">
+        <v>4600</v>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D43" s="23" t="inlineStr">
+        <is>
+          <t>S00498</t>
+        </is>
+      </c>
+      <c r="E43" s="23" t="inlineStr">
+        <is>
+          <t>CONTROL</t>
+        </is>
+      </c>
+      <c r="F43" s="24" t="n">
+        <v>46189</v>
+      </c>
+      <c r="G43" s="24" t="n">
+        <v>46190.87469875543</v>
+      </c>
+      <c r="H43" t="inlineStr">
+        <is>
+          <t>NS</t>
+        </is>
+      </c>
+      <c r="J43" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="K43" s="25" t="n">
+        <v>82100</v>
+      </c>
+      <c r="BS43" t="n">
+        <v>4600</v>
+      </c>
+      <c r="BT43" t="inlineStr">
+        <is>
+          <t>51000100</t>
+        </is>
+      </c>
+      <c r="BU43" s="23" t="inlineStr">
+        <is>
+          <t>Supplies</t>
+        </is>
+      </c>
+      <c r="BV43" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="BW43" s="25" t="n">
+        <v>82100</v>
+      </c>
+      <c r="BX43" t="inlineStr">
+        <is>
+          <t>I0</t>
+        </is>
+      </c>
+      <c r="BY43" t="inlineStr"/>
+      <c r="CA43" t="inlineStr">
+        <is>
+          <t>460020450</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="n">
+        <v>38</v>
+      </c>
+      <c r="B44" t="n">
+        <v>4600</v>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D44" s="23" t="inlineStr">
+        <is>
+          <t>V00055</t>
+        </is>
+      </c>
+      <c r="E44" s="23" t="inlineStr">
+        <is>
+          <t>207753428</t>
+        </is>
+      </c>
+      <c r="F44" s="24" t="n">
+        <v>46149</v>
+      </c>
+      <c r="G44" s="24" t="n">
+        <v>46190.87469876715</v>
+      </c>
+      <c r="H44" t="inlineStr">
+        <is>
+          <t>NS</t>
+        </is>
+      </c>
+      <c r="J44" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="K44" s="25" t="n">
+        <v>829.98</v>
+      </c>
+      <c r="BS44" t="n">
+        <v>4600</v>
+      </c>
+      <c r="BT44" t="inlineStr">
+        <is>
+          <t>51000100</t>
+        </is>
+      </c>
+      <c r="BU44" s="23" t="inlineStr">
+        <is>
+          <t>Supplies</t>
+        </is>
+      </c>
+      <c r="BV44" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="BW44" s="25" t="n">
+        <v>829.98</v>
+      </c>
+      <c r="BX44" t="inlineStr">
+        <is>
+          <t>I0</t>
+        </is>
+      </c>
+      <c r="BY44" t="inlineStr"/>
+      <c r="CA44" t="inlineStr">
+        <is>
+          <t>460020450</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="n">
+        <v>39</v>
+      </c>
+      <c r="B45" t="n">
+        <v>4600</v>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D45" s="23" t="inlineStr">
+        <is>
+          <t>V02263</t>
+        </is>
+      </c>
+      <c r="E45" s="23" t="inlineStr">
+        <is>
+          <t>1152787-IN</t>
+        </is>
+      </c>
+      <c r="F45" s="24" t="n">
+        <v>46176</v>
+      </c>
+      <c r="G45" s="24" t="n">
+        <v>46190.87469876715</v>
+      </c>
+      <c r="H45" t="inlineStr">
+        <is>
+          <t>NS</t>
+        </is>
+      </c>
+      <c r="J45" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="K45" s="25" t="n">
+        <v>1093.44</v>
+      </c>
+      <c r="BS45" t="n">
+        <v>4600</v>
+      </c>
+      <c r="BT45" t="inlineStr">
+        <is>
+          <t>51000100</t>
+        </is>
+      </c>
+      <c r="BU45" s="23" t="inlineStr">
+        <is>
+          <t>Supplies</t>
+        </is>
+      </c>
+      <c r="BV45" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="BW45" s="25" t="n">
+        <v>1093.44</v>
+      </c>
+      <c r="BX45" t="inlineStr">
+        <is>
+          <t>I0</t>
+        </is>
+      </c>
+      <c r="BY45" t="inlineStr"/>
+      <c r="CA45" t="inlineStr">
+        <is>
+          <t>460020450</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="n">
+        <v>40</v>
+      </c>
+      <c r="B46" t="n">
+        <v>4600</v>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D46" s="23" t="inlineStr">
+        <is>
+          <t>V08728</t>
+        </is>
+      </c>
+      <c r="E46" s="23" t="inlineStr">
+        <is>
+          <t>9807-R1</t>
+        </is>
+      </c>
+      <c r="F46" s="24" t="n">
+        <v>46189</v>
+      </c>
+      <c r="G46" s="24" t="n">
+        <v>46190.87469876715</v>
+      </c>
+      <c r="H46" t="inlineStr">
+        <is>
+          <t>NS</t>
+        </is>
+      </c>
+      <c r="J46" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="K46" s="25" t="n">
+        <v>100</v>
+      </c>
+      <c r="BS46" t="n">
+        <v>4600</v>
+      </c>
+      <c r="BT46" t="inlineStr">
+        <is>
+          <t>51000100</t>
+        </is>
+      </c>
+      <c r="BU46" s="23" t="inlineStr">
+        <is>
+          <t>Supplies</t>
+        </is>
+      </c>
+      <c r="BV46" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="BW46" s="25" t="n">
+        <v>100</v>
+      </c>
+      <c r="BX46" t="inlineStr">
+        <is>
+          <t>I0</t>
+        </is>
+      </c>
+      <c r="BY46" t="inlineStr"/>
+      <c r="CA46" t="inlineStr">
+        <is>
+          <t>460020450</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="n">
+        <v>41</v>
+      </c>
+      <c r="B47" t="n">
+        <v>4600</v>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D47" s="23" t="inlineStr">
+        <is>
+          <t>V04415</t>
+        </is>
+      </c>
+      <c r="E47" s="23" t="inlineStr">
+        <is>
+          <t>29647</t>
+        </is>
+      </c>
+      <c r="F47" s="24" t="n">
+        <v>46189</v>
+      </c>
+      <c r="G47" s="24" t="n">
+        <v>46190.87469876715</v>
+      </c>
+      <c r="H47" t="inlineStr">
+        <is>
+          <t>NS</t>
+        </is>
+      </c>
+      <c r="J47" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="K47" s="25" t="n">
+        <v>4800</v>
+      </c>
+      <c r="BS47" t="n">
+        <v>4600</v>
+      </c>
+      <c r="BT47" t="inlineStr">
+        <is>
+          <t>51000100</t>
+        </is>
+      </c>
+      <c r="BU47" s="23" t="inlineStr">
+        <is>
+          <t>Supplies</t>
+        </is>
+      </c>
+      <c r="BV47" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="BW47" s="25" t="n">
+        <v>4800</v>
+      </c>
+      <c r="BX47" t="inlineStr">
+        <is>
+          <t>I0</t>
+        </is>
+      </c>
+      <c r="BY47" t="inlineStr"/>
+      <c r="CA47" t="inlineStr">
+        <is>
+          <t>460020450</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="n">
+        <v>42</v>
+      </c>
+      <c r="B48" t="n">
+        <v>4600</v>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D48" s="23" t="inlineStr">
+        <is>
+          <t>V01706</t>
+        </is>
+      </c>
+      <c r="E48" s="23" t="inlineStr">
+        <is>
+          <t>300000372</t>
+        </is>
+      </c>
+      <c r="F48" s="24" t="n">
+        <v>46173</v>
+      </c>
+      <c r="G48" s="24" t="n">
+        <v>46190.87469876715</v>
+      </c>
+      <c r="H48" t="inlineStr">
+        <is>
+          <t>NS</t>
+        </is>
+      </c>
+      <c r="J48" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="K48" s="25" t="n">
+        <v>38.4</v>
+      </c>
+      <c r="BS48" t="n">
+        <v>4600</v>
+      </c>
+      <c r="BT48" t="inlineStr">
+        <is>
+          <t>51000100</t>
+        </is>
+      </c>
+      <c r="BU48" s="23" t="inlineStr">
+        <is>
+          <t>Supplies</t>
+        </is>
+      </c>
+      <c r="BV48" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="BW48" s="25" t="n">
+        <v>38.4</v>
+      </c>
+      <c r="BX48" t="inlineStr">
+        <is>
+          <t>I0</t>
+        </is>
+      </c>
+      <c r="BY48" t="inlineStr"/>
+      <c r="CA48" t="inlineStr">
         <is>
           <t>460020450</t>
         </is>

</xml_diff>